<commit_message>
chore(data): refresh bundled workbook with Value Framework + Value Trees sheets
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/app/excel/strategy.xlsx
+++ b/server/app/excel/strategy.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30203"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/riccardo.lana/Projects/MFG/v3/assets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wppcloud.sharepoint.com/sites/WT-P-U-Growth/Shared Documents/Active pitches/Google/Google Media Workflow Agentification/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3AB391C4-F688-2D4C-B28D-D15B89B0CF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{959D68C4-734A-43B6-B148-D5056BE45D81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{09DA6218-4145-413E-8449-5E430392F1AB}"/>
+    <workbookView xWindow="13995" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="3" xr2:uid="{09DA6218-4145-413E-8449-5E430392F1AB}"/>
   </bookViews>
   <sheets>
     <sheet name="JTBD" sheetId="1" r:id="rId1"/>
     <sheet name="Overview MFG enablers " sheetId="6" r:id="rId2"/>
+    <sheet name="Value Framework" sheetId="8" r:id="rId3"/>
+    <sheet name="Value Trees" sheetId="7" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1016" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1175" uniqueCount="663">
   <si>
     <t>Phase</t>
   </si>
@@ -2433,12 +2435,294 @@
   <si>
     <t>Derives parallel structures from other industries to de-risk adoption of new media strategies</t>
   </si>
+  <si>
+    <t xml:space="preserve">Phase </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value dimension </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimension definition </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimension used in phase? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Key opportunities </t>
+  </si>
+  <si>
+    <t>Shared opportunity?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KPIs </t>
+  </si>
+  <si>
+    <t>Effectiveness</t>
+  </si>
+  <si>
+    <t>Effectiveness: Sharpen strategic hypotheses and strengthen recommendation quality by proactively surfacing historical learnings against benchmarks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automated Historical Learnings Synthesis </t>
+  </si>
+  <si>
+    <t>% campaigns with learnings at inception · Repeat-mistake ↓%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Execution </t>
+  </si>
+  <si>
+    <t>Execution: Scale institutional knowledge across 1,500+ people and markets, enabling self-serve access without dependency on individual handoffs.</t>
+  </si>
+  <si>
+    <t>Growth Opportunity Surfacing</t>
+  </si>
+  <si>
+    <t>Hypotheses/qtr · Acceptance % · Performance lift %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Efficiency </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Efficiency: Reduce manual data assembly and accelerate insight generation by unifying fragmented sources into a persistent intelligence layer. </t>
+  </si>
+  <si>
+    <t>Dynamic Product Insights Access</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes </t>
+  </si>
+  <si>
+    <t>% plans with product context overlaid · Relevance score Δ</t>
+  </si>
+  <si>
+    <t>Cross-PA Knowledge Sharing at Scale</t>
+  </si>
+  <si>
+    <t>Monthly active users · Self-serve resolution %</t>
+  </si>
+  <si>
+    <t>Connected Research Infrastructure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assembly productivity ↑% · Sources unified into single layer </t>
+  </si>
+  <si>
+    <t>Automated Strategy-to-Production Handoff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Days strategy→brief · Manual steps eliminated </t>
+  </si>
+  <si>
+    <t>Live Scenario Planning Capability</t>
+  </si>
+  <si>
+    <t>Modelling responsiveness ↑ · Scenarios per cycle ↑</t>
+  </si>
+  <si>
+    <t>Effectiveness: Improve plan quality and creative accuracy by standardizing formats and reducing specification errors across Product Areas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No </t>
+  </si>
+  <si>
+    <t>Standardized Asset Tracker Across Product Areas</t>
+  </si>
+  <si>
+    <t>PAs on unified format % · Spec error rate ↓%</t>
+  </si>
+  <si>
+    <t>Execution: Enable agencies and teams to self-serve on best practices and standards, reducing dependency on repeated manual education.</t>
+  </si>
+  <si>
+    <t>Automated Tactical Data Assembly</t>
+  </si>
+  <si>
+    <t>Manual re-keys eliminated</t>
+  </si>
+  <si>
+    <t>Efficiency: Eliminate manual re-keying in plan assembly and compress planning timelines through automated data unification and linked documents.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linked Scenario Plan and CAP </t>
+  </si>
+  <si>
+    <t>Sync productivity ↑% · Update propagation responsiveness ↑</t>
+  </si>
+  <si>
+    <t>Digital Best Practices Self-Service</t>
+  </si>
+  <si>
+    <t>Self-serve resolution % · Briefing productivity ↑</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Activate </t>
+  </si>
+  <si>
+    <t>Effectiveness: Raise QA coverage and improve launch quality through systematic governance, ensuring measurement alignment before builds begin.</t>
+  </si>
+  <si>
+    <t>Campaign Governance as the QA Backbone</t>
+  </si>
+  <si>
+    <t>% campaigns through CG · QA coverage %</t>
+  </si>
+  <si>
+    <t>Execution: Create a consistent, scalable monitoring standard across PAs by consolidating ~60 dashboards into one unified platform.</t>
+  </si>
+  <si>
+    <t>Measurement &amp; Test Alignment at Setup</t>
+  </si>
+  <si>
+    <t>% locked at scenario approval · Delay days ↓</t>
+  </si>
+  <si>
+    <t>Efficiency: Reduce rework and accelerate pre-launch validation by catching defects earlier before they cascade across vendor platforms.</t>
+  </si>
+  <si>
+    <t>Consolidated Monitoring (~60 to 1)</t>
+  </si>
+  <si>
+    <t>Dashboards consolidated · % reporting via OMS</t>
+  </si>
+  <si>
+    <t>Reducing Rework from Upstream Quality</t>
+  </si>
+  <si>
+    <t>Defects caught at trafficking stage % · Rework ↓</t>
+  </si>
+  <si>
+    <t>Effectiveness: Establish trust in central data through visible integrity metrics, making platform-direct pulls the exception rather than the default.</t>
+  </si>
+  <si>
+    <t>Accountability Infrastructure for Data Compliance</t>
+  </si>
+  <si>
+    <t>% reporting via central platform · Data trust score %</t>
+  </si>
+  <si>
+    <t>Execution: Improve stakeholder confidence through governance OKRs, escalation paths, and a knowledge layer that makes the right action obvious.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consolidate Data Visibility </t>
+  </si>
+  <si>
+    <t>Dashboards consolidated · Remediation responsiveness ↑</t>
+  </si>
+  <si>
+    <t>Efficiency: Reduce duplicated oversight effort by consolidating fragmented data integrity dashboards into a single view with clear remediation guidance.</t>
+  </si>
+  <si>
+    <t>Bypassed Central Infrastructure</t>
+  </si>
+  <si>
+    <t>Compliance OKR attainment % · Stakeholder confidence score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value Framework legend </t>
+  </si>
+  <si>
+    <t xml:space="preserve">title </t>
+  </si>
+  <si>
+    <t xml:space="preserve">definition </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value dimensions </t>
+  </si>
+  <si>
+    <t>Which dimensions drive value in this phase?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What are the key initiatives that are going to drive value in this phase? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value dimensions definition </t>
+  </si>
+  <si>
+    <t xml:space="preserve">What does each value dimension mean in this phase? </t>
+  </si>
+  <si>
+    <t>KPIs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How are we going to measure success? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value dimensions  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enablers </t>
+  </si>
+  <si>
+    <t>#04.17 Goldfoil</t>
+  </si>
+  <si>
+    <t>#01.16 Strategy Weaver (Agent)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#01.02 Audience Insights </t>
+  </si>
+  <si>
+    <t>Execution</t>
+  </si>
+  <si>
+    <t>#01.17 SLA &amp; Blueprint Navigator (Agent)</t>
+  </si>
+  <si>
+    <t>Efficiency</t>
+  </si>
+  <si>
+    <t>#01.01 Strategic Insights
+#01.07 Charm</t>
+  </si>
+  <si>
+    <t>#01.02  Audience Insights 
+#02.02 Campaign Tactics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#02.01 Campaign Strategies </t>
+  </si>
+  <si>
+    <t>#02.08 Google Sheets (Asset Tracker)</t>
+  </si>
+  <si>
+    <t>#02.01 Campaign Tactics</t>
+  </si>
+  <si>
+    <t>#04.01 Buttery Dashboard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#03.01 Campaign Governance </t>
+  </si>
+  <si>
+    <t>#04.02 MFG App</t>
+  </si>
+  <si>
+    <t>#04.05 Campaign Performance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#03.01 Campaign Governance
+#03.03 Creative Analytics </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyze </t>
+  </si>
+  <si>
+    <t>#05.05 Campaign Mgmt (Olive) Helper (Agent)</t>
+  </si>
+  <si>
+    <t>#04.08 Data Integrity</t>
+  </si>
+  <si>
+    <t>#04.06 DataLab / EMDP</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2461,8 +2745,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2475,8 +2774,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -2484,11 +2789,63 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2552,6 +2909,37 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="20" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2566,6 +2954,15 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2925,25 +3322,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5E0576A-B5F4-4D7C-92F8-73DCFEFA83D4}">
   <dimension ref="A1:Q37"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="10.5" customWidth="1"/>
-    <col min="2" max="2" width="34.83203125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="45.33203125" style="6" customWidth="1"/>
-    <col min="4" max="4" width="86.5" style="6" customWidth="1"/>
-    <col min="5" max="5" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" customWidth="1"/>
+    <col min="2" max="2" width="34.85546875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="45.28515625" style="6" customWidth="1"/>
+    <col min="4" max="4" width="86.5703125" style="6" customWidth="1"/>
+    <col min="5" max="5" width="28.85546875" customWidth="1"/>
     <col min="6" max="6" width="40" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.6640625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="21.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="24.85546875" customWidth="1"/>
     <col min="9" max="9" width="26" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="25.83203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="29.6640625" customWidth="1"/>
-    <col min="14" max="16" width="27.1640625" customWidth="1"/>
-    <col min="17" max="17" width="36.83203125" customWidth="1"/>
+    <col min="10" max="10" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="29.7109375" customWidth="1"/>
+    <col min="14" max="16" width="27.140625" customWidth="1"/>
+    <col min="17" max="17" width="36.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:17">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="11" t="s">
@@ -2955,49 +3352,49 @@
       <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="26" t="s">
+      <c r="E1" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="26" t="s">
+      <c r="F1" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="27" t="s">
+      <c r="G1" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="26" t="s">
+      <c r="H1" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="26" t="s">
+      <c r="I1" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="26" t="s">
+      <c r="J1" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="25" t="s">
+      <c r="K1" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25" t="s">
+      <c r="L1" s="38"/>
+      <c r="M1" s="38"/>
+      <c r="N1" s="38" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="25"/>
-      <c r="P1" s="25"/>
+      <c r="O1" s="38"/>
+      <c r="P1" s="38"/>
       <c r="Q1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A2" s="26"/>
+    <row r="2" spans="1:17">
+      <c r="A2" s="39"/>
       <c r="B2" s="11"/>
       <c r="C2" s="12"/>
       <c r="D2" s="12"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="39"/>
+      <c r="I2" s="39"/>
+      <c r="J2" s="39"/>
       <c r="K2" s="1" t="s">
         <v>13</v>
       </c>
@@ -3017,17 +3414,17 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:17" ht="136.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" ht="136.5" customHeight="1">
       <c r="A3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="36" t="s">
         <v>19</v>
       </c>
       <c r="E3" s="4" t="s">
@@ -3067,13 +3464,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:17" s="3" customFormat="1" ht="240" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" s="3" customFormat="1" ht="217.5">
       <c r="A4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="23"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
+      <c r="B4" s="36"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
       <c r="E4" s="4" t="s">
         <v>30</v>
       </c>
@@ -3111,13 +3508,13 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="3" customFormat="1" ht="256" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" s="3" customFormat="1" ht="231.95">
       <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="23"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="36"/>
       <c r="E5" s="4" t="s">
         <v>41</v>
       </c>
@@ -3155,13 +3552,13 @@
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:17" s="3" customFormat="1" ht="224" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" s="3" customFormat="1" ht="203.1">
       <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="36"/>
       <c r="E6" s="4" t="s">
         <v>52</v>
       </c>
@@ -3199,13 +3596,13 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:17" s="3" customFormat="1" ht="32" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" s="3" customFormat="1" ht="29.1">
       <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="23"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="23"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
       <c r="E7" s="4" t="s">
         <v>61</v>
       </c>
@@ -3243,17 +3640,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:17" s="3" customFormat="1" ht="245.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" s="3" customFormat="1" ht="245.25" customHeight="1">
       <c r="A8" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="37" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="37" t="s">
         <v>71</v>
       </c>
       <c r="E8" s="20" t="s">
@@ -3294,13 +3691,13 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:17" s="3" customFormat="1" ht="144" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" s="3" customFormat="1" ht="130.5">
       <c r="A9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
       <c r="E9" s="7" t="s">
         <v>83</v>
       </c>
@@ -3338,13 +3735,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:17" s="3" customFormat="1" ht="128" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" s="3" customFormat="1" ht="116.1">
       <c r="A10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="37"/>
+      <c r="D10" s="37"/>
       <c r="E10" s="4" t="s">
         <v>92</v>
       </c>
@@ -3382,13 +3779,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:17" s="3" customFormat="1" ht="96" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" s="3" customFormat="1" ht="101.45">
       <c r="A11" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
+      <c r="B11" s="37"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="37"/>
       <c r="E11" s="4" t="s">
         <v>103</v>
       </c>
@@ -3426,13 +3823,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:17" s="3" customFormat="1" ht="144" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" s="3" customFormat="1" ht="130.5">
       <c r="A12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
+      <c r="B12" s="37"/>
+      <c r="C12" s="37"/>
+      <c r="D12" s="37"/>
       <c r="E12" s="4" t="s">
         <v>111</v>
       </c>
@@ -3470,13 +3867,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:17" s="3" customFormat="1" ht="128" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" s="3" customFormat="1" ht="116.1">
       <c r="A13" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
       <c r="E13" s="4" t="s">
         <v>119</v>
       </c>
@@ -3514,13 +3911,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:17" s="3" customFormat="1" ht="144" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" s="3" customFormat="1" ht="130.5">
       <c r="A14" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="37"/>
+      <c r="D14" s="37"/>
       <c r="E14" s="4" t="s">
         <v>127</v>
       </c>
@@ -3558,13 +3955,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:17" s="3" customFormat="1" ht="208" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" s="3" customFormat="1" ht="188.45">
       <c r="A15" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
+      <c r="B15" s="37"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="37"/>
       <c r="E15" s="4" t="s">
         <v>135</v>
       </c>
@@ -3602,17 +3999,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:17" s="3" customFormat="1" ht="256" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" s="3" customFormat="1" ht="261">
       <c r="A16" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="B16" s="24" t="s">
+      <c r="B16" s="37" t="s">
         <v>145</v>
       </c>
-      <c r="C16" s="24" t="s">
+      <c r="C16" s="37" t="s">
         <v>146</v>
       </c>
-      <c r="D16" s="24" t="s">
+      <c r="D16" s="37" t="s">
         <v>147</v>
       </c>
       <c r="E16" s="16" t="s">
@@ -3655,13 +4052,13 @@
         <v>159</v>
       </c>
     </row>
-    <row r="17" spans="1:17" s="3" customFormat="1" ht="176" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17" s="3" customFormat="1" ht="174">
       <c r="A17" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
       <c r="E17" s="14" t="s">
         <v>160</v>
       </c>
@@ -3699,13 +4096,13 @@
         <v>168</v>
       </c>
     </row>
-    <row r="18" spans="1:17" s="3" customFormat="1" ht="176" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:17" s="3" customFormat="1" ht="159.6">
       <c r="A18" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
       <c r="E18" s="14" t="s">
         <v>169</v>
       </c>
@@ -3743,17 +4140,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:17" s="3" customFormat="1" ht="160" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:17" s="3" customFormat="1" ht="144.94999999999999">
       <c r="A19" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="B19" s="23" t="s">
+      <c r="B19" s="36" t="s">
         <v>177</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="36" t="s">
         <v>178</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" s="36" t="s">
         <v>179</v>
       </c>
       <c r="E19" s="14" t="s">
@@ -3793,13 +4190,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:17" s="3" customFormat="1" ht="176" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:17" s="3" customFormat="1" ht="188.45">
       <c r="A20" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
       <c r="E20" s="14" t="s">
         <v>190</v>
       </c>
@@ -3837,13 +4234,13 @@
         <v>198</v>
       </c>
     </row>
-    <row r="21" spans="1:17" s="3" customFormat="1" ht="112" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:17" s="3" customFormat="1" ht="101.45">
       <c r="A21" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="36"/>
+      <c r="D21" s="36"/>
       <c r="E21" s="14" t="s">
         <v>199</v>
       </c>
@@ -3881,7 +4278,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:17" s="3" customFormat="1" ht="267.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:17" s="3" customFormat="1" ht="267.75" customHeight="1">
       <c r="A22" s="15" t="s">
         <v>144</v>
       </c>
@@ -3934,17 +4331,17 @@
         <v>223</v>
       </c>
     </row>
-    <row r="23" spans="1:17" s="3" customFormat="1" ht="160" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:17" s="3" customFormat="1" ht="159.6">
       <c r="A23" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="36" t="s">
         <v>225</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C23" s="36" t="s">
         <v>226</v>
       </c>
-      <c r="D23" s="23" t="s">
+      <c r="D23" s="36" t="s">
         <v>227</v>
       </c>
       <c r="E23" s="4" t="s">
@@ -3984,13 +4381,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:17" s="3" customFormat="1" ht="160" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:17" s="3" customFormat="1" ht="144.94999999999999">
       <c r="A24" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="B24" s="23"/>
-      <c r="C24" s="23"/>
-      <c r="D24" s="23"/>
+      <c r="B24" s="36"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
       <c r="E24" s="14" t="s">
         <v>238</v>
       </c>
@@ -4028,13 +4425,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="25" spans="1:17" s="3" customFormat="1" ht="192" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:17" s="3" customFormat="1" ht="174">
       <c r="A25" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="23"/>
-      <c r="D25" s="23"/>
+      <c r="B25" s="36"/>
+      <c r="C25" s="36"/>
+      <c r="D25" s="36"/>
       <c r="E25" s="14" t="s">
         <v>247</v>
       </c>
@@ -4072,13 +4469,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="26" spans="1:17" s="3" customFormat="1" ht="176" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:17" s="3" customFormat="1" ht="174">
       <c r="A26" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="B26" s="23"/>
-      <c r="C26" s="23"/>
-      <c r="D26" s="23"/>
+      <c r="B26" s="36"/>
+      <c r="C26" s="36"/>
+      <c r="D26" s="36"/>
       <c r="E26" s="14" t="s">
         <v>256</v>
       </c>
@@ -4116,13 +4513,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="27" spans="1:17" s="3" customFormat="1" ht="144" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:17" s="3" customFormat="1" ht="144.94999999999999">
       <c r="A27" s="15" t="s">
         <v>224</v>
       </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
+      <c r="B27" s="36"/>
+      <c r="C27" s="36"/>
+      <c r="D27" s="36"/>
       <c r="E27" s="16" t="s">
         <v>265</v>
       </c>
@@ -4163,13 +4560,13 @@
         <v>275</v>
       </c>
     </row>
-    <row r="28" spans="1:17" s="3" customFormat="1" ht="144" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:17" s="3" customFormat="1" ht="130.5">
       <c r="A28" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="B28" s="23"/>
-      <c r="C28" s="23"/>
-      <c r="D28" s="23"/>
+      <c r="B28" s="36"/>
+      <c r="C28" s="36"/>
+      <c r="D28" s="36"/>
       <c r="E28" s="14" t="s">
         <v>276</v>
       </c>
@@ -4207,17 +4604,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:17" s="3" customFormat="1" ht="192" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:17" s="3" customFormat="1" ht="217.5">
       <c r="A29" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="B29" s="23" t="s">
+      <c r="B29" s="36" t="s">
         <v>285</v>
       </c>
-      <c r="C29" s="23" t="s">
+      <c r="C29" s="36" t="s">
         <v>286</v>
       </c>
-      <c r="D29" s="23" t="s">
+      <c r="D29" s="36" t="s">
         <v>287</v>
       </c>
       <c r="E29" s="14" t="s">
@@ -4257,13 +4654,13 @@
         <v>296</v>
       </c>
     </row>
-    <row r="30" spans="1:17" s="3" customFormat="1" ht="176" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:17" s="3" customFormat="1" ht="159.6">
       <c r="A30" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="B30" s="23"/>
-      <c r="C30" s="23"/>
-      <c r="D30" s="23"/>
+      <c r="B30" s="36"/>
+      <c r="C30" s="36"/>
+      <c r="D30" s="36"/>
       <c r="E30" s="14" t="s">
         <v>297</v>
       </c>
@@ -4301,17 +4698,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="31" spans="1:17" s="3" customFormat="1" ht="160" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:17" s="3" customFormat="1" ht="144.94999999999999">
       <c r="A31" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="B31" s="23" t="s">
+      <c r="B31" s="36" t="s">
         <v>306</v>
       </c>
-      <c r="C31" s="23" t="s">
+      <c r="C31" s="36" t="s">
         <v>307</v>
       </c>
-      <c r="D31" s="23" t="s">
+      <c r="D31" s="36" t="s">
         <v>308</v>
       </c>
       <c r="E31" s="14" t="s">
@@ -4351,13 +4748,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:17" s="3" customFormat="1" ht="160" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:17" s="3" customFormat="1" ht="159.6">
       <c r="A32" s="15" t="s">
         <v>305</v>
       </c>
-      <c r="B32" s="23"/>
-      <c r="C32" s="23"/>
-      <c r="D32" s="23"/>
+      <c r="B32" s="36"/>
+      <c r="C32" s="36"/>
+      <c r="D32" s="36"/>
       <c r="E32" s="16" t="s">
         <v>319</v>
       </c>
@@ -4398,13 +4795,13 @@
         <v>329</v>
       </c>
     </row>
-    <row r="33" spans="1:16" s="3" customFormat="1" ht="176" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" s="3" customFormat="1" ht="159.6">
       <c r="A33" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="B33" s="23"/>
-      <c r="C33" s="23"/>
-      <c r="D33" s="23"/>
+      <c r="B33" s="36"/>
+      <c r="C33" s="36"/>
+      <c r="D33" s="36"/>
       <c r="E33" s="14" t="s">
         <v>330</v>
       </c>
@@ -4442,13 +4839,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="1:16" s="3" customFormat="1" ht="160" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16" s="3" customFormat="1" ht="159.6">
       <c r="A34" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="B34" s="23"/>
-      <c r="C34" s="23"/>
-      <c r="D34" s="23"/>
+      <c r="B34" s="36"/>
+      <c r="C34" s="36"/>
+      <c r="D34" s="36"/>
       <c r="E34" s="14" t="s">
         <v>338</v>
       </c>
@@ -4486,17 +4883,17 @@
         <v>347</v>
       </c>
     </row>
-    <row r="35" spans="1:16" s="3" customFormat="1" ht="192" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" s="3" customFormat="1" ht="174">
       <c r="A35" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="B35" s="23" t="s">
+      <c r="B35" s="36" t="s">
         <v>348</v>
       </c>
-      <c r="C35" s="23" t="s">
+      <c r="C35" s="36" t="s">
         <v>349</v>
       </c>
-      <c r="D35" s="23" t="s">
+      <c r="D35" s="36" t="s">
         <v>350</v>
       </c>
       <c r="E35" s="14" t="s">
@@ -4536,13 +4933,13 @@
         <v>359</v>
       </c>
     </row>
-    <row r="36" spans="1:16" s="3" customFormat="1" ht="240" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" s="3" customFormat="1" ht="217.5">
       <c r="A36" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="B36" s="23"/>
-      <c r="C36" s="23"/>
-      <c r="D36" s="23"/>
+      <c r="B36" s="36"/>
+      <c r="C36" s="36"/>
+      <c r="D36" s="36"/>
       <c r="E36" s="14" t="s">
         <v>360</v>
       </c>
@@ -4580,13 +4977,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="37" spans="1:16" s="3" customFormat="1" ht="304" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16" s="3" customFormat="1" ht="275.45">
       <c r="A37" s="3" t="s">
         <v>305</v>
       </c>
-      <c r="B37" s="23"/>
-      <c r="C37" s="23"/>
-      <c r="D37" s="23"/>
+      <c r="B37" s="36"/>
+      <c r="C37" s="36"/>
+      <c r="D37" s="36"/>
       <c r="E37" s="14" t="s">
         <v>369</v>
       </c>
@@ -4667,17 +5064,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF7A1A4-7C00-4F8E-ACF6-178DE6D0EA93}">
   <dimension ref="A1:G85"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" style="1"/>
-    <col min="2" max="2" width="36.83203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" customWidth="1"/>
-    <col min="6" max="6" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="86.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="60.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="2" max="2" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="23.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="86.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="60.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>377</v>
       </c>
@@ -4700,7 +5097,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7">
       <c r="A2" s="22">
         <v>4.2361111111111113E-2</v>
       </c>
@@ -4723,7 +5120,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7">
       <c r="A3" s="22">
         <v>4.3055555555555555E-2</v>
       </c>
@@ -4746,7 +5143,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7">
       <c r="A4" s="22">
         <v>4.3749999999999997E-2</v>
       </c>
@@ -4769,7 +5166,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7">
       <c r="A5" s="22">
         <v>4.4444444444444446E-2</v>
       </c>
@@ -4792,7 +5189,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7">
       <c r="A6" s="22">
         <v>4.5138888888888888E-2</v>
       </c>
@@ -4815,7 +5212,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7">
       <c r="A7" s="22">
         <v>4.583333333333333E-2</v>
       </c>
@@ -4838,7 +5235,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7">
       <c r="A8" s="22">
         <v>4.6527777777777779E-2</v>
       </c>
@@ -4861,7 +5258,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7">
       <c r="A9" s="22">
         <v>4.7222222222222221E-2</v>
       </c>
@@ -4884,7 +5281,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7">
       <c r="A10" s="22">
         <v>4.791666666666667E-2</v>
       </c>
@@ -4907,7 +5304,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7">
       <c r="A11" s="22">
         <v>4.8611111111111112E-2</v>
       </c>
@@ -4930,7 +5327,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7">
       <c r="A12" s="22">
         <v>4.9305555555555554E-2</v>
       </c>
@@ -4953,7 +5350,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7">
       <c r="A13" s="22">
         <v>0.05</v>
       </c>
@@ -4976,7 +5373,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7">
       <c r="A14" s="22">
         <v>5.0694444444444445E-2</v>
       </c>
@@ -4999,7 +5396,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7">
       <c r="A15" s="22">
         <v>5.1388888888888887E-2</v>
       </c>
@@ -5022,7 +5419,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7">
       <c r="A16" s="22">
         <v>5.2083333333333336E-2</v>
       </c>
@@ -5045,7 +5442,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7">
       <c r="A17" s="22">
         <v>5.2777777777777778E-2</v>
       </c>
@@ -5068,7 +5465,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7">
       <c r="A18" s="22">
         <v>5.347222222222222E-2</v>
       </c>
@@ -5091,7 +5488,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7">
       <c r="A19" s="22">
         <v>5.4166666666666669E-2</v>
       </c>
@@ -5114,7 +5511,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7">
       <c r="A20" s="22">
         <v>5.486111111111111E-2</v>
       </c>
@@ -5137,7 +5534,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7">
       <c r="A21" s="22">
         <v>5.5555555555555552E-2</v>
       </c>
@@ -5160,7 +5557,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7">
       <c r="A22" s="22">
         <v>5.6250000000000001E-2</v>
       </c>
@@ -5183,7 +5580,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:7">
       <c r="A23" s="22">
         <v>5.6944444444444443E-2</v>
       </c>
@@ -5206,7 +5603,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7">
       <c r="A24" s="22">
         <v>5.7638888888888892E-2</v>
       </c>
@@ -5229,7 +5626,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7">
       <c r="A25" s="22">
         <v>5.8333333333333334E-2</v>
       </c>
@@ -5252,7 +5649,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7">
       <c r="A26" s="22">
         <v>5.9027777777777776E-2</v>
       </c>
@@ -5275,7 +5672,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7">
       <c r="A27" s="22">
         <v>5.9722222222222225E-2</v>
       </c>
@@ -5298,7 +5695,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7">
       <c r="A28" s="22">
         <v>6.0416666666666667E-2</v>
       </c>
@@ -5321,7 +5718,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7">
       <c r="A29" s="22">
         <v>6.1111111111111109E-2</v>
       </c>
@@ -5344,7 +5741,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7">
       <c r="A30" s="22">
         <v>6.1805555555555558E-2</v>
       </c>
@@ -5367,7 +5764,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7">
       <c r="A31" s="22">
         <v>6.25E-2</v>
       </c>
@@ -5390,7 +5787,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7">
       <c r="A32" s="22">
         <v>6.3194444444444442E-2</v>
       </c>
@@ -5413,7 +5810,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7">
       <c r="A33" s="22">
         <v>6.3888888888888884E-2</v>
       </c>
@@ -5436,7 +5833,7 @@
         <v>457</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7">
       <c r="A34" s="22">
         <v>8.4027777777777785E-2</v>
       </c>
@@ -5459,7 +5856,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7">
       <c r="A35" s="22">
         <v>8.4722222222222227E-2</v>
       </c>
@@ -5482,7 +5879,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7">
       <c r="A36" s="22">
         <v>8.5416666666666669E-2</v>
       </c>
@@ -5505,7 +5902,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7">
       <c r="A37" s="22">
         <v>8.611111111111111E-2</v>
       </c>
@@ -5528,7 +5925,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7">
       <c r="A38" s="22">
         <v>8.6805555555555552E-2</v>
       </c>
@@ -5551,7 +5948,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7">
       <c r="A39" s="22">
         <v>8.7499999999999994E-2</v>
       </c>
@@ -5574,7 +5971,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7">
       <c r="A40" s="22">
         <v>8.819444444444445E-2</v>
       </c>
@@ -5597,7 +5994,7 @@
         <v>473</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7">
       <c r="A41" s="22">
         <v>8.8888888888888892E-2</v>
       </c>
@@ -5620,7 +6017,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7">
       <c r="A42" s="22">
         <v>8.9583333333333334E-2</v>
       </c>
@@ -5643,7 +6040,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7">
       <c r="A43" s="22">
         <v>9.0277777777777776E-2</v>
       </c>
@@ -5666,7 +6063,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7">
       <c r="A44" s="22">
         <v>9.0972222222222218E-2</v>
       </c>
@@ -5689,7 +6086,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7">
       <c r="A45" s="22">
         <v>9.166666666666666E-2</v>
       </c>
@@ -5712,7 +6109,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7">
       <c r="A46" s="22">
         <v>0.12569444444444444</v>
       </c>
@@ -5735,7 +6132,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7">
       <c r="A47" s="22">
         <v>0.12638888888888888</v>
       </c>
@@ -5758,7 +6155,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:7">
       <c r="A48" s="22">
         <v>0.12708333333333333</v>
       </c>
@@ -5781,7 +6178,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7">
       <c r="A49" s="22">
         <v>0.12777777777777777</v>
       </c>
@@ -5804,7 +6201,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7">
       <c r="A50" s="22">
         <v>0.12847222222222221</v>
       </c>
@@ -5827,7 +6224,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7">
       <c r="A51" s="22">
         <v>0.12916666666666668</v>
       </c>
@@ -5850,7 +6247,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7">
       <c r="A52" s="22">
         <v>0.12986111111111112</v>
       </c>
@@ -5873,7 +6270,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7">
       <c r="A53" s="22">
         <v>0.13055555555555556</v>
       </c>
@@ -5896,7 +6293,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:7">
       <c r="A54" s="22">
         <v>0.13125000000000001</v>
       </c>
@@ -5919,7 +6316,7 @@
         <v>502</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7">
       <c r="A55" s="22">
         <v>0.13194444444444445</v>
       </c>
@@ -5942,7 +6339,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7">
       <c r="A56" s="22">
         <v>0.13263888888888889</v>
       </c>
@@ -5965,7 +6362,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7">
       <c r="A57" s="22">
         <v>0.13333333333333333</v>
       </c>
@@ -5988,7 +6385,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7">
       <c r="A58" s="22">
         <v>0.13402777777777777</v>
       </c>
@@ -6011,7 +6408,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7">
       <c r="A59" s="22">
         <v>0.13472222222222222</v>
       </c>
@@ -6034,7 +6431,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7">
       <c r="A60" s="22">
         <v>0.13541666666666666</v>
       </c>
@@ -6057,7 +6454,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7">
       <c r="A61" s="22">
         <v>0.1673611111111111</v>
       </c>
@@ -6080,7 +6477,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7">
       <c r="A62" s="22">
         <v>0.16805555555555557</v>
       </c>
@@ -6103,7 +6500,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7">
       <c r="A63" s="22">
         <v>0.16875000000000001</v>
       </c>
@@ -6126,7 +6523,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7">
       <c r="A64" s="22">
         <v>0.16944444444444445</v>
       </c>
@@ -6149,7 +6546,7 @@
         <v>525</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7">
       <c r="A65" s="22">
         <v>0.1701388888888889</v>
       </c>
@@ -6172,7 +6569,7 @@
         <v>526</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:7">
       <c r="A66" s="22">
         <v>0.17083333333333334</v>
       </c>
@@ -6195,7 +6592,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7">
       <c r="A67" s="22">
         <v>0.17152777777777778</v>
       </c>
@@ -6218,7 +6615,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:7">
       <c r="A68" s="22">
         <v>0.17222222222222222</v>
       </c>
@@ -6241,7 +6638,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7">
       <c r="A69" s="22">
         <v>0.17291666666666666</v>
       </c>
@@ -6264,7 +6661,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7">
       <c r="A70" s="22">
         <v>0.1736111111111111</v>
       </c>
@@ -6287,7 +6684,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7">
       <c r="A71" s="22">
         <v>0.17430555555555555</v>
       </c>
@@ -6310,7 +6707,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7">
       <c r="A72" s="22">
         <v>0.17499999999999999</v>
       </c>
@@ -6333,7 +6730,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:7">
       <c r="A73" s="22">
         <v>0.17569444444444443</v>
       </c>
@@ -6356,7 +6753,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7">
       <c r="A74" s="22">
         <v>0.1763888888888889</v>
       </c>
@@ -6379,7 +6776,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7">
       <c r="A75" s="22">
         <v>0.17708333333333334</v>
       </c>
@@ -6402,7 +6799,7 @@
         <v>546</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7">
       <c r="A76" s="22">
         <v>0.17777777777777778</v>
       </c>
@@ -6425,7 +6822,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:7">
       <c r="A77" s="22">
         <v>0.17847222222222223</v>
       </c>
@@ -6448,7 +6845,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:7">
       <c r="A78" s="22">
         <v>0.17916666666666667</v>
       </c>
@@ -6471,7 +6868,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7">
       <c r="A79" s="22">
         <v>0.17986111111111111</v>
       </c>
@@ -6494,7 +6891,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7">
       <c r="A80" s="22">
         <v>0.20902777777777778</v>
       </c>
@@ -6517,7 +6914,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:7">
       <c r="A81" s="22">
         <v>0.20972222222222223</v>
       </c>
@@ -6540,7 +6937,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7">
       <c r="A82" s="22">
         <v>0.21041666666666667</v>
       </c>
@@ -6563,7 +6960,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:7">
       <c r="A83" s="22">
         <v>0.21111111111111111</v>
       </c>
@@ -6586,7 +6983,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:7">
       <c r="A84" s="22">
         <v>0.21180555555555555</v>
       </c>
@@ -6609,7 +7006,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:7">
       <c r="A85" s="22">
         <v>0.21249999999999999</v>
       </c>
@@ -6640,28 +7037,709 @@
 </worksheet>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <MigrationWizIdSecurityGroups xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <MigrationWizIdPermissions xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
-    <TaxCatchAll xmlns="c7a2b444-66b6-41fc-9d77-e176b311c743" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <MigrationWizIdDocumentLibraryPermissions xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
-    <MigrationWizIdPermissionLevels xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Growthtags xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
-    <Relevant xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
-    <MigrationWizId xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
-    <Archived xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2">false</Archived>
-  </documentManagement>
-</p:properties>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84D6C7FC-1B5C-420E-BC9B-00532D37E354}">
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
+  <cols>
+    <col min="1" max="1" width="10.85546875" customWidth="1"/>
+    <col min="2" max="2" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="4" max="4" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.42578125" style="34" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="54" style="34" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="26" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>571</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>572</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>573</v>
+      </c>
+      <c r="E1" s="30" t="s">
+        <v>574</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>575</v>
+      </c>
+      <c r="G1" s="30" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="70.5" customHeight="1">
+      <c r="A2" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>577</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>578</v>
+      </c>
+      <c r="D2" s="25"/>
+      <c r="E2" s="31" t="s">
+        <v>579</v>
+      </c>
+      <c r="F2" s="24"/>
+      <c r="G2" s="31" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="87.6" customHeight="1">
+      <c r="A3" s="35"/>
+      <c r="B3" s="24" t="s">
+        <v>581</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>582</v>
+      </c>
+      <c r="D3" s="25"/>
+      <c r="E3" s="31" t="s">
+        <v>583</v>
+      </c>
+      <c r="F3" s="24"/>
+      <c r="G3" s="31" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="91.5" customHeight="1">
+      <c r="A4" s="35"/>
+      <c r="B4" s="24" t="s">
+        <v>585</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>586</v>
+      </c>
+      <c r="D4" s="25"/>
+      <c r="E4" s="31" t="s">
+        <v>587</v>
+      </c>
+      <c r="F4" s="24" t="s">
+        <v>588</v>
+      </c>
+      <c r="G4" s="31" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="35"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="31" t="s">
+        <v>590</v>
+      </c>
+      <c r="F5" s="24"/>
+      <c r="G5" s="31" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="35"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="31" t="s">
+        <v>592</v>
+      </c>
+      <c r="F6" s="24"/>
+      <c r="G6" s="31" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="35"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="31" t="s">
+        <v>594</v>
+      </c>
+      <c r="F7" s="24"/>
+      <c r="G7" s="31" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="35"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="31" t="s">
+        <v>596</v>
+      </c>
+      <c r="F8" s="24"/>
+      <c r="G8" s="31" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="57.95">
+      <c r="A9" s="35" t="s">
+        <v>144</v>
+      </c>
+      <c r="B9" s="24" t="s">
+        <v>577</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>598</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>599</v>
+      </c>
+      <c r="E9" s="31" t="s">
+        <v>600</v>
+      </c>
+      <c r="F9" s="24"/>
+      <c r="G9" s="31" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="57.95">
+      <c r="A10" s="35"/>
+      <c r="B10" s="24" t="s">
+        <v>581</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>602</v>
+      </c>
+      <c r="D10" s="25"/>
+      <c r="E10" s="31" t="s">
+        <v>603</v>
+      </c>
+      <c r="F10" s="24"/>
+      <c r="G10" s="31" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="57.95">
+      <c r="A11" s="35"/>
+      <c r="B11" s="24" t="s">
+        <v>585</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>605</v>
+      </c>
+      <c r="D11" s="25"/>
+      <c r="E11" s="31" t="s">
+        <v>606</v>
+      </c>
+      <c r="F11" s="24"/>
+      <c r="G11" s="31" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="35"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="31" t="s">
+        <v>608</v>
+      </c>
+      <c r="F12" s="24"/>
+      <c r="G12" s="31" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="72.599999999999994">
+      <c r="A13" s="35" t="s">
+        <v>610</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>577</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>611</v>
+      </c>
+      <c r="D13" s="24"/>
+      <c r="E13" s="31" t="s">
+        <v>612</v>
+      </c>
+      <c r="F13" s="24"/>
+      <c r="G13" s="31" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="57.95">
+      <c r="A14" s="35"/>
+      <c r="B14" s="24" t="s">
+        <v>581</v>
+      </c>
+      <c r="C14" s="25" t="s">
+        <v>614</v>
+      </c>
+      <c r="D14" s="24"/>
+      <c r="E14" s="31" t="s">
+        <v>615</v>
+      </c>
+      <c r="F14" s="24" t="s">
+        <v>588</v>
+      </c>
+      <c r="G14" s="31" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="57.95">
+      <c r="A15" s="35"/>
+      <c r="B15" s="24" t="s">
+        <v>585</v>
+      </c>
+      <c r="C15" s="25" t="s">
+        <v>617</v>
+      </c>
+      <c r="D15" s="24"/>
+      <c r="E15" s="31" t="s">
+        <v>618</v>
+      </c>
+      <c r="F15" s="24"/>
+      <c r="G15" s="31" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="35"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="31" t="s">
+        <v>620</v>
+      </c>
+      <c r="F16" s="24"/>
+      <c r="G16" s="31" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="57.95">
+      <c r="A17" s="41" t="s">
+        <v>305</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>577</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>622</v>
+      </c>
+      <c r="D17" s="24"/>
+      <c r="E17" s="32" t="s">
+        <v>623</v>
+      </c>
+      <c r="F17" s="24"/>
+      <c r="G17" s="31" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="57.95">
+      <c r="A18" s="42"/>
+      <c r="B18" s="24" t="s">
+        <v>581</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>625</v>
+      </c>
+      <c r="D18" s="24"/>
+      <c r="E18" s="31" t="s">
+        <v>626</v>
+      </c>
+      <c r="F18" s="24"/>
+      <c r="G18" s="31" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="57.95">
+      <c r="A19" s="43"/>
+      <c r="B19" s="24" t="s">
+        <v>585</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>628</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>599</v>
+      </c>
+      <c r="E19" s="33" t="s">
+        <v>629</v>
+      </c>
+      <c r="F19" s="24"/>
+      <c r="G19" s="31" t="s">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="26" t="s">
+        <v>631</v>
+      </c>
+      <c r="B23" s="29"/>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="1" t="s">
+        <v>632</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="57.95">
+      <c r="A25" s="2" t="s">
+        <v>634</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="72.599999999999994">
+      <c r="A26" s="2" t="s">
+        <v>574</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="57.95">
+      <c r="A27" s="2" t="s">
+        <v>637</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="43.5">
+      <c r="A28" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="2"/>
+      <c r="B29" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:A8"/>
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="A13:A16"/>
+    <mergeCell ref="A17:A19"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D4A9EE1-232A-445B-8BFE-B287909575EB}">
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
+  <cols>
+    <col min="2" max="2" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="54" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1">
+      <c r="A1" s="26" t="s">
+        <v>570</v>
+      </c>
+      <c r="B1" s="26" t="s">
+        <v>641</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>574</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>642</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="35" t="s">
+        <v>577</v>
+      </c>
+      <c r="C2" s="24" t="s">
+        <v>579</v>
+      </c>
+      <c r="D2" s="24" t="s">
+        <v>643</v>
+      </c>
+      <c r="E2" s="24" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="35"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="24" t="s">
+        <v>583</v>
+      </c>
+      <c r="D3" s="24" t="s">
+        <v>644</v>
+      </c>
+      <c r="E3" s="24" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="35"/>
+      <c r="B4" s="35"/>
+      <c r="C4" s="24" t="s">
+        <v>587</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>645</v>
+      </c>
+      <c r="E4" s="24" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="35"/>
+      <c r="B5" s="23" t="s">
+        <v>646</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>590</v>
+      </c>
+      <c r="D5" s="24" t="s">
+        <v>647</v>
+      </c>
+      <c r="E5" s="24" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="29.1">
+      <c r="A6" s="35"/>
+      <c r="B6" s="35" t="s">
+        <v>648</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>592</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>649</v>
+      </c>
+      <c r="E6" s="24" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="29.1">
+      <c r="A7" s="35"/>
+      <c r="B7" s="35"/>
+      <c r="C7" s="24" t="s">
+        <v>594</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>650</v>
+      </c>
+      <c r="E7" s="24" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="35"/>
+      <c r="B8" s="35"/>
+      <c r="C8" s="24" t="s">
+        <v>596</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>651</v>
+      </c>
+      <c r="E8" s="24" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="35" t="s">
+        <v>144</v>
+      </c>
+      <c r="B9" s="23" t="s">
+        <v>581</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>600</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>652</v>
+      </c>
+      <c r="E9" s="24" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="35"/>
+      <c r="B10" s="35" t="s">
+        <v>585</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>603</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>653</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="35"/>
+      <c r="B11" s="35"/>
+      <c r="C11" s="24" t="s">
+        <v>606</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>654</v>
+      </c>
+      <c r="E11" s="24" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="35"/>
+      <c r="B12" s="35"/>
+      <c r="C12" s="24" t="s">
+        <v>608</v>
+      </c>
+      <c r="D12" s="24" t="s">
+        <v>647</v>
+      </c>
+      <c r="E12" s="24" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="35" t="s">
+        <v>224</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>577</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>612</v>
+      </c>
+      <c r="D13" s="24" t="s">
+        <v>655</v>
+      </c>
+      <c r="E13" s="24" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="35"/>
+      <c r="B14" s="35" t="s">
+        <v>646</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>615</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>656</v>
+      </c>
+      <c r="E14" s="24" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="35"/>
+      <c r="B15" s="35"/>
+      <c r="C15" s="24" t="s">
+        <v>618</v>
+      </c>
+      <c r="D15" s="24" t="s">
+        <v>657</v>
+      </c>
+      <c r="E15" s="24" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="29.1">
+      <c r="A16" s="35"/>
+      <c r="B16" s="23" t="s">
+        <v>648</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>620</v>
+      </c>
+      <c r="D16" s="25" t="s">
+        <v>658</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="35" t="s">
+        <v>659</v>
+      </c>
+      <c r="B17" s="23" t="s">
+        <v>581</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>623</v>
+      </c>
+      <c r="D17" s="24" t="s">
+        <v>660</v>
+      </c>
+      <c r="E17" s="24" t="s">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="35"/>
+      <c r="B18" s="35" t="s">
+        <v>577</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>626</v>
+      </c>
+      <c r="D18" s="24" t="s">
+        <v>661</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="35"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="28" t="s">
+        <v>629</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>662</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>630</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A17:A19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B2:B4"/>
+    <mergeCell ref="B6:B8"/>
+    <mergeCell ref="A2:A8"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="A13:A16"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005CBA3BB114BFD74789BBC2112E83CA05" ma:contentTypeVersion="30" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b2807d0a8b93919cc076dad061ecb86f">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="bf98a0ff-8200-4e6b-9275-c8b7c887382e" xmlns:ns3="835b0495-f08e-41df-93b5-9f7800c83c0d" xmlns:ns4="034baa58-2ee9-40c3-871d-a6d8878677e2" xmlns:ns5="c7a2b444-66b6-41fc-9d77-e176b311c743" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4e39cd897662b439ab7c55dc7c6b390e" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -7019,7 +8097,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -7028,52 +8106,35 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <MigrationWizIdSecurityGroups xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <MigrationWizIdPermissions xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
+    <TaxCatchAll xmlns="c7a2b444-66b6-41fc-9d77-e176b311c743" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <MigrationWizIdDocumentLibraryPermissions xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
+    <MigrationWizIdPermissionLevels xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Growthtags xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
+    <Relevant xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
+    <MigrationWizId xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2" xsi:nil="true"/>
+    <Archived xmlns="034baa58-2ee9-40c3-871d-a6d8878677e2">false</Archived>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC74B1A8-5C46-4750-AA98-FE51890F63E2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="034baa58-2ee9-40c3-871d-a6d8878677e2"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="c7a2b444-66b6-41fc-9d77-e176b311c743"/>
-    <ds:schemaRef ds:uri="835b0495-f08e-41df-93b5-9f7800c83c0d"/>
-    <ds:schemaRef ds:uri="bf98a0ff-8200-4e6b-9275-c8b7c887382e"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEE69217-B4E5-45F7-8430-CA485B62A03C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DEE69217-B4E5-45F7-8430-CA485B62A03C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="bf98a0ff-8200-4e6b-9275-c8b7c887382e"/>
-    <ds:schemaRef ds:uri="835b0495-f08e-41df-93b5-9f7800c83c0d"/>
-    <ds:schemaRef ds:uri="034baa58-2ee9-40c3-871d-a6d8878677e2"/>
-    <ds:schemaRef ds:uri="c7a2b444-66b6-41fc-9d77-e176b311c743"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6286E33-1708-465F-8F81-E63F2FA7BF4C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6286E33-1708-465F-8F81-E63F2FA7BF4C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC74B1A8-5C46-4750-AA98-FE51890F63E2}"/>
 </file>
</xml_diff>